<commit_message>
Update Zergaw_territory_ranking_chart with updated work
</commit_message>
<xml_diff>
--- a/Zergaw_territory_ranking_chart.xlsx
+++ b/Zergaw_territory_ranking_chart.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tihitinazergaw\Documents\DATA_Labs\Capstone_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{65675C93-BE79-4BDF-B2F0-A0F2F6244A85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7E06014-ED8B-44EA-891A-D53C018CAA0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{3F04257C-D03E-4537-AC2E-EB3138680232}"/>
   </bookViews>
@@ -17,13 +17,13 @@
   </sheets>
   <calcPr calcId="0"/>
   <pivotCaches>
-    <pivotCache cacheId="5" r:id="rId2"/>
+    <pivotCache cacheId="0" r:id="rId2"/>
   </pivotCaches>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="5">
   <si>
     <t>TotalSales</t>
   </si>
@@ -35,6 +35,9 @@
   </si>
   <si>
     <t>Total Sales</t>
+  </si>
+  <si>
+    <t>Store 853 has higher total sales than store 852 by 25,191.44</t>
   </si>
 </sst>
 </file>
@@ -518,9 +521,8 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -677,6 +679,47 @@
         <c:marker>
           <c:symbol val="none"/>
         </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
       </c:pivotFmt>
     </c:pivotFmts>
     <c:plotArea>
@@ -745,7 +788,6 @@
           </c:extLst>
         </c:ser>
         <c:dLbls>
-          <c:dLblPos val="outEnd"/>
           <c:showLegendKey val="0"/>
           <c:showVal val="0"/>
           <c:showCatName val="0"/>
@@ -1569,7 +1611,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FF3379F3-C8AF-49C5-B0CF-83EEE065576A}" name="PivotTable1" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Store_ID">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FF3379F3-C8AF-49C5-B0CF-83EEE065576A}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Store_ID">
   <location ref="D2:E5" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="2">
     <pivotField dataField="1" showAll="0"/>
@@ -1941,7 +1983,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21044E55-39DE-4F20-A7A8-66F9B8621B54}">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.81640625" bestFit="1" customWidth="1"/>
@@ -1966,7 +2008,7 @@
       <c r="B2">
         <v>852</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="E2" t="s">
@@ -1980,27 +2022,32 @@
       <c r="B3">
         <v>853</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="2">
         <v>852</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3">
         <v>311810.56</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="D4" s="3">
+      <c r="D4" s="2">
         <v>853</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4">
         <v>337002</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5">
         <v>648812.56000000006</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>